<commit_message>
introduced tutorial jupyter Notebook
</commit_message>
<xml_diff>
--- a/SHARC_tests.xlsx
+++ b/SHARC_tests.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smhhborg\Desktop\test for SHARC Crosswalks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\smhhborg(D_Laufwerk)\Documents\GitHub\test_for_shacl_shape_bridges\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11850" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11850"/>
   </bookViews>
   <sheets>
     <sheet name="Curies" sheetId="1" r:id="rId1"/>
@@ -184,16 +184,16 @@
     <t>Specimen</t>
   </si>
   <si>
-    <t>class_label</t>
-  </si>
-  <si>
-    <t>class_curie</t>
-  </si>
-  <si>
     <t>relation_label</t>
   </si>
   <si>
     <t>relation_curie</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>curie</t>
   </si>
 </sst>
 </file>
@@ -524,16 +524,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>53</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>